<commit_message>
Modificaciones para excel segun el dia
</commit_message>
<xml_diff>
--- a/facultad-derecho/tempExcels/Semana1.xlsx
+++ b/facultad-derecho/tempExcels/Semana1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet sheetId="6" name="ASIGNACIÓN TURNOS" state="visible" r:id="rId4"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1311" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="286">
   <si>
     <t>UNIVERSIDAD COLEGIO MAYOR DE CUNDINAMARCA</t>
   </si>
@@ -739,7 +739,7 @@
     <t>LISTADO DE ASIGNACION DE TURNOS PARA ESTUDIANTES  PERIODO  2025-II</t>
   </si>
   <si>
-    <t>SEMANA No. 7 SEPTIEMBRE 08-12</t>
+    <t>SEMANA No. 17 NOVIEMBRE 19 - 21</t>
   </si>
   <si>
     <t>APELLIDOS Y NOMBRES ESTUDIANTE</t>
@@ -766,79 +766,94 @@
     <t xml:space="preserve">LUNES </t>
   </si>
   <si>
-    <t>JUL-28,-2025</t>
-  </si>
-  <si>
     <t>LINA PAOLA TRIANA MARTINEZ</t>
   </si>
   <si>
-    <t>RUIZ SAENZ JUANA MARIA</t>
-  </si>
-  <si>
     <t>ROBERTO ANGEL BADRAN BLANCO</t>
   </si>
   <si>
-    <t>SUAREZ MURCIA DUVAN STIVEN</t>
+    <t>ERICK SANTIAGO RICO LOPEZ</t>
+  </si>
+  <si>
+    <t>MIERCOLES</t>
+  </si>
+  <si>
+    <t>NOV-19,-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANDRES RICARDO MORENO SANGUINO </t>
+  </si>
+  <si>
+    <t>DAVID RICARDO JARAMILLO ZALDUA</t>
+  </si>
+  <si>
+    <t>FRANCISCO ALVARO FAJARDO PINILLA</t>
+  </si>
+  <si>
+    <t>PAULA ANDREA QUINTERO VARGAS</t>
   </si>
   <si>
     <t>MORALES PERALTA VALENTINA</t>
   </si>
   <si>
+    <t>LEIDY NATALIA MONCADA VEGA</t>
+  </si>
+  <si>
+    <t>WILLIAM GIOVANNI MORENO AVILA</t>
+  </si>
+  <si>
+    <t>DANIEL ESTEBAN QUINTERO CARMONA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JUEVES </t>
+  </si>
+  <si>
+    <t>JAIME ESTEBAN CAMARGO MENA</t>
+  </si>
+  <si>
+    <t>NOV-20,-2025</t>
+  </si>
+  <si>
+    <t>ROSEMBER SIERRA AVILA</t>
+  </si>
+  <si>
+    <t>SANTIAGO GONZALEZ VARGAS</t>
+  </si>
+  <si>
+    <t>KAROL ANDREA FLOREZ RODRIGUEZ</t>
+  </si>
+  <si>
+    <t>NICOL DAYAN JIMENEZ GUTIERREZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JONIER ALEXANDER ROJAS </t>
+  </si>
+  <si>
+    <t>VIERNES</t>
+  </si>
+  <si>
+    <t>NOV-21,-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROCIO DEL PILAR ROJAS ROCHA </t>
+  </si>
+  <si>
+    <t>TANIA SOFIA RAMIREZ MEDINA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NELSON ENRIQUE RUEDA RODRIGUEZ </t>
+  </si>
+  <si>
+    <t>KIMBERLY DANIELA GONZALES CARRERO</t>
+  </si>
+  <si>
+    <t>JIMENEZ GALVIS ISIDRO</t>
+  </si>
+  <si>
+    <t>JULIAN ESTEBAN ACERO CASTILLO</t>
+  </si>
+  <si>
     <t>DÍA DE CONCILIACIONES Y/O SALIDA PEDAGOGICA</t>
-  </si>
-  <si>
-    <t>SANCHEZ MOTTA LAURA SOFÍA</t>
-  </si>
-  <si>
-    <t>MIERCOLES</t>
-  </si>
-  <si>
-    <t>JUL-30,-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANDRES RICARDO MORENO SANGUINO </t>
-  </si>
-  <si>
-    <t>FRANCISCO ALVARO FAJARDO PINILLA</t>
-  </si>
-  <si>
-    <t>ALISON LOPEZ</t>
-  </si>
-  <si>
-    <t>WILLIAM GIOVANNI MORENO AVILA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUEVES </t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEVIN JULIAN CAMILO ESPITIA RINCON </t>
-  </si>
-  <si>
-    <t>JUL-31,-2025</t>
-  </si>
-  <si>
-    <t>ROSEMBER SIERRA AVILA</t>
-  </si>
-  <si>
-    <t>JIMENEZ ALFONSO TATIANA</t>
-  </si>
-  <si>
-    <t>VIERNES</t>
-  </si>
-  <si>
-    <t>AUG-01,-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROCIO DEL PILAR ROJAS ROCHA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">NELSON ENRIQUE RUEDA RODRIGUEZ </t>
-  </si>
-  <si>
-    <t>ANA MARIA VILLALBA SUAREZ</t>
-  </si>
-  <si>
-    <t>SERRATO SOTO JANA VALENTINA</t>
   </si>
   <si>
     <t xml:space="preserve">MODIFICACION  DE TURNOS </t>
@@ -1070,7 +1085,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -1425,6 +1440,89 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.3999755851924192"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.3999755851924192"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1446,50 +1544,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1814,6 +1873,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1840,87 +1902,102 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2332,18 +2409,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J38"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.42578125"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="11.453125" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" customWidth="1"/>
-    <col min="2" max="2" width="43.140625" style="109" customWidth="1"/>
-    <col min="3" max="3" width="5.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" customWidth="1"/>
+    <col min="2" max="2" width="43.1796875" style="109" customWidth="1"/>
+    <col min="3" max="3" width="5.1796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
-    <col min="7" max="7" width="24.42578125" customWidth="1"/>
-    <col min="8" max="8" width="46.85546875" customWidth="1"/>
-    <col min="9" max="9" width="31.42578125" customWidth="1"/>
-    <col min="10" max="10" width="22.7109375" customWidth="1"/>
+    <col min="6" max="6" width="9.54296875" customWidth="1"/>
+    <col min="7" max="7" width="24.453125" customWidth="1"/>
+    <col min="8" max="8" width="46.81640625" customWidth="1"/>
+    <col min="9" max="9" width="31.453125" customWidth="1"/>
+    <col min="10" max="10" width="22.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
@@ -2455,211 +2532,223 @@
     </row>
     <row r="8" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="124"/>
-      <c r="B8" s="125" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="126">
-        <v>3</v>
-      </c>
+      <c r="B8" s="125"/>
+      <c r="C8" s="126"/>
       <c r="D8" s="126" t="s">
         <v>247</v>
       </c>
-      <c r="E8" s="127" t="s">
-        <v>248</v>
-      </c>
-      <c r="F8" s="126" t="s">
-        <v>15</v>
-      </c>
+      <c r="E8" s="127"/>
+      <c r="F8" s="126"/>
       <c r="G8" s="128"/>
       <c r="H8" s="129" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I8" s="130"/>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="131"/>
-      <c r="B9" s="23" t="s">
-        <v>250</v>
-      </c>
-      <c r="C9" s="24">
-        <v>2</v>
-      </c>
+      <c r="B9" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="24"/>
       <c r="D9" s="24"/>
-      <c r="E9" s="46" t="s">
-        <v>248</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>15</v>
-      </c>
+      <c r="E9" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="F9" s="24"/>
       <c r="G9" s="25"/>
       <c r="H9" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="I9" s="132"/>
-    </row>
-    <row r="10" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>248</v>
+      </c>
+      <c r="I9" s="133"/>
+    </row>
+    <row r="10" ht="15.5" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="131"/>
-      <c r="B10" s="23"/>
+      <c r="B10" s="132" t="s">
+        <v>160</v>
+      </c>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
-      <c r="E10" s="46"/>
+      <c r="E10" s="132" t="s">
+        <v>160</v>
+      </c>
       <c r="F10" s="24"/>
       <c r="G10" s="25"/>
       <c r="H10" s="23" t="s">
-        <v>251</v>
-      </c>
-      <c r="I10" s="132"/>
-    </row>
-    <row r="11" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>249</v>
+      </c>
+      <c r="I10" s="133"/>
+    </row>
+    <row r="11" ht="15.5" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="131"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="133"/>
+      <c r="B11" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="C11" s="134"/>
       <c r="D11" s="24"/>
-      <c r="E11" s="46"/>
+      <c r="E11" s="132" t="s">
+        <v>160</v>
+      </c>
       <c r="F11" s="24"/>
       <c r="G11" s="25"/>
       <c r="H11" s="28"/>
-      <c r="I11" s="132"/>
-    </row>
-    <row r="12" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I11" s="133"/>
+    </row>
+    <row r="12" ht="15.5" customHeight="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="131"/>
-      <c r="B12" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="C12" s="24">
-        <v>3</v>
-      </c>
+      <c r="B12" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="C12" s="24"/>
       <c r="D12" s="24"/>
-      <c r="E12" s="46" t="s">
-        <v>248</v>
-      </c>
-      <c r="F12" s="24" t="s">
-        <v>20</v>
-      </c>
+      <c r="E12" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="F12" s="24"/>
       <c r="G12" s="25"/>
       <c r="H12" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="I12" s="132"/>
-      <c r="J12" s="134"/>
-    </row>
-    <row r="13" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I12" s="133"/>
+      <c r="J12" s="135"/>
+    </row>
+    <row r="13" ht="15.5" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="131"/>
-      <c r="B13" s="23" t="s">
-        <v>253</v>
-      </c>
-      <c r="C13" s="24">
-        <v>4</v>
-      </c>
+      <c r="B13" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="C13" s="24"/>
       <c r="D13" s="24"/>
-      <c r="E13" s="46" t="s">
-        <v>248</v>
-      </c>
-      <c r="F13" s="24" t="s">
-        <v>20</v>
-      </c>
+      <c r="E13" s="132" t="s">
+        <v>160</v>
+      </c>
+      <c r="F13" s="24"/>
       <c r="G13" s="25"/>
       <c r="H13" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="I13" s="132"/>
+        <v>248</v>
+      </c>
+      <c r="I13" s="133"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="135"/>
-      <c r="B14" s="136"/>
-      <c r="C14" s="137"/>
-      <c r="D14" s="137"/>
-      <c r="E14" s="138"/>
-      <c r="F14" s="137"/>
-      <c r="G14" s="139"/>
-      <c r="H14" s="140" t="s">
-        <v>249</v>
-      </c>
-      <c r="I14" s="141"/>
-    </row>
-    <row r="15" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="142" t="s">
+      <c r="A14" s="136"/>
+      <c r="B14" s="137"/>
+      <c r="C14" s="138"/>
+      <c r="D14" s="138"/>
+      <c r="E14" s="139"/>
+      <c r="F14" s="138"/>
+      <c r="G14" s="140"/>
+      <c r="H14" s="141" t="s">
+        <v>248</v>
+      </c>
+      <c r="I14" s="142"/>
+    </row>
+    <row r="15" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="124"/>
+      <c r="B15" s="143" t="s">
+        <v>250</v>
+      </c>
+      <c r="C15" s="144">
+        <v>1</v>
+      </c>
+      <c r="D15" s="145" t="s">
+        <v>251</v>
+      </c>
+      <c r="E15" s="127" t="s">
+        <v>252</v>
+      </c>
+      <c r="F15" s="126" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="128"/>
+      <c r="H15" s="129" t="s">
+        <v>253</v>
+      </c>
+      <c r="I15" s="130"/>
+    </row>
+    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="131"/>
+      <c r="B16" s="23" t="s">
         <v>254</v>
       </c>
-      <c r="B15" s="143"/>
-      <c r="C15" s="143"/>
-      <c r="D15" s="143"/>
-      <c r="E15" s="143"/>
-      <c r="F15" s="143"/>
-      <c r="G15" s="143"/>
-      <c r="H15" s="143"/>
-      <c r="I15" s="144"/>
-    </row>
-    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="124"/>
-      <c r="B16" s="145" t="s">
+      <c r="C16" s="24">
+        <v>4</v>
+      </c>
+      <c r="D16" s="146"/>
+      <c r="E16" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="F16" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="25"/>
+      <c r="H16" s="23" t="s">
         <v>255</v>
       </c>
-      <c r="C16" s="146">
-        <v>1</v>
-      </c>
-      <c r="D16" s="147" t="s">
-        <v>256</v>
-      </c>
-      <c r="E16" s="127" t="s">
-        <v>257</v>
-      </c>
-      <c r="F16" s="126" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" s="128"/>
-      <c r="H16" s="129" t="s">
-        <v>258</v>
-      </c>
-      <c r="I16" s="130"/>
+      <c r="I16" s="133"/>
     </row>
     <row r="17" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="131"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="148"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="24"/>
+      <c r="B17" s="52" t="s">
+        <v>256</v>
+      </c>
+      <c r="C17" s="24">
+        <v>3</v>
+      </c>
+      <c r="D17" s="146"/>
+      <c r="E17" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="F17" s="24" t="s">
+        <v>15</v>
+      </c>
       <c r="G17" s="25"/>
       <c r="H17" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="I17" s="132"/>
+        <v>255</v>
+      </c>
+      <c r="I17" s="133"/>
     </row>
     <row r="18" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="131"/>
-      <c r="B18" s="52"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="148"/>
-      <c r="E18" s="46"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="134"/>
+      <c r="D18" s="146"/>
       <c r="F18" s="24"/>
       <c r="G18" s="25"/>
-      <c r="H18" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="I18" s="132"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="133"/>
     </row>
     <row r="19" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="131"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="133"/>
-      <c r="D19" s="148"/>
-      <c r="F19" s="24"/>
+      <c r="B19" s="72" t="s">
+        <v>257</v>
+      </c>
+      <c r="C19" s="24">
+        <v>4</v>
+      </c>
+      <c r="D19" s="146"/>
+      <c r="E19" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>20</v>
+      </c>
       <c r="G19" s="25"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="132"/>
+      <c r="H19" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="I19" s="133"/>
     </row>
     <row r="20" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="131"/>
-      <c r="B20" s="72" t="s">
-        <v>260</v>
-      </c>
-      <c r="C20" s="24">
-        <v>2</v>
-      </c>
-      <c r="D20" s="148"/>
+      <c r="B20" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="C20" s="55">
+        <v>4</v>
+      </c>
+      <c r="D20" s="146"/>
       <c r="E20" s="46" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="F20" s="24" t="s">
         <v>20</v>
@@ -2668,296 +2757,336 @@
       <c r="H20" s="23" t="s">
         <v>259</v>
       </c>
-      <c r="I20" s="132"/>
-    </row>
-    <row r="21" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="131"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="55"/>
+      <c r="I20" s="133"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="136"/>
+      <c r="B21" s="77" t="s">
+        <v>260</v>
+      </c>
+      <c r="C21" s="147">
+        <v>4</v>
+      </c>
       <c r="D21" s="148"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="25"/>
+      <c r="E21" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="F21" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="G21" s="140"/>
       <c r="H21" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="I21" s="142"/>
+    </row>
+    <row r="22" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="124"/>
+      <c r="B22" s="149"/>
+      <c r="C22" s="126"/>
+      <c r="D22" s="150" t="s">
         <v>261</v>
       </c>
-      <c r="I21" s="132"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="135"/>
-      <c r="B22" s="77"/>
-      <c r="C22" s="149"/>
-      <c r="D22" s="150"/>
-      <c r="E22" s="138"/>
-      <c r="F22" s="137"/>
-      <c r="G22" s="139"/>
-      <c r="H22" s="23" t="s">
-        <v>261</v>
-      </c>
-      <c r="I22" s="141"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="126"/>
+      <c r="G22" s="126"/>
+      <c r="H22" s="129"/>
+      <c r="I22" s="130"/>
     </row>
     <row r="23" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="124"/>
-      <c r="B23" s="151"/>
-      <c r="C23" s="126"/>
-      <c r="D23" s="152" t="s">
+      <c r="A23" s="152"/>
+      <c r="B23" s="52" t="s">
         <v>262</v>
       </c>
-      <c r="E23" s="153"/>
-      <c r="F23" s="126"/>
-      <c r="G23" s="126"/>
-      <c r="H23" s="129"/>
-      <c r="I23" s="130"/>
+      <c r="C23" s="24">
+        <v>1</v>
+      </c>
+      <c r="D23" s="67"/>
+      <c r="E23" s="46" t="s">
+        <v>263</v>
+      </c>
+      <c r="F23" s="67" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="71"/>
+      <c r="H23" s="52" t="s">
+        <v>264</v>
+      </c>
+      <c r="I23" s="153"/>
     </row>
     <row r="24" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="154"/>
-      <c r="B24" s="52" t="s">
-        <v>263</v>
-      </c>
-      <c r="C24" s="24">
-        <v>3</v>
+      <c r="A24" s="152"/>
+      <c r="B24" s="31" t="s">
+        <v>265</v>
+      </c>
+      <c r="C24" s="38">
+        <v>1</v>
       </c>
       <c r="D24" s="67"/>
       <c r="E24" s="46" t="s">
+        <v>263</v>
+      </c>
+      <c r="F24" s="67" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="68"/>
+      <c r="H24" s="52" t="s">
         <v>264</v>
       </c>
-      <c r="F24" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="71"/>
-      <c r="H24" s="52" t="s">
-        <v>265</v>
-      </c>
-      <c r="I24" s="155"/>
+      <c r="I24" s="153"/>
     </row>
     <row r="25" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="154"/>
-      <c r="B25" s="31" t="s">
+      <c r="A25" s="152"/>
+      <c r="B25" s="125" t="s">
         <v>266</v>
       </c>
-      <c r="C25" s="38">
+      <c r="C25" s="55">
+        <v>2</v>
+      </c>
+      <c r="D25" s="67"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="71"/>
+      <c r="H25" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" s="153"/>
+    </row>
+    <row r="26" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="152"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="67"/>
+      <c r="G26" s="67"/>
+      <c r="H26" s="154"/>
+      <c r="I26" s="153"/>
+    </row>
+    <row r="27" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="152"/>
+      <c r="B27" s="77" t="s">
+        <v>267</v>
+      </c>
+      <c r="C27" s="24">
         <v>4</v>
       </c>
-      <c r="D25" s="67"/>
-      <c r="E25" s="46" t="s">
-        <v>264</v>
-      </c>
-      <c r="F25" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" s="68"/>
-      <c r="H25" s="52" t="s">
-        <v>265</v>
-      </c>
-      <c r="I25" s="155"/>
-    </row>
-    <row r="26" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="154"/>
-      <c r="B26" s="125"/>
-      <c r="C26" s="55"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="46"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="71"/>
-      <c r="H26" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="I26" s="155"/>
-    </row>
-    <row r="27" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="154"/>
-      <c r="B27" s="26"/>
-      <c r="C27" s="24"/>
       <c r="D27" s="67"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="156"/>
-      <c r="I27" s="155"/>
+      <c r="E27" s="46" t="s">
+        <v>263</v>
+      </c>
+      <c r="F27" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27" s="71"/>
+      <c r="H27" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="I27" s="153"/>
     </row>
     <row r="28" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="154"/>
-      <c r="B28" s="52"/>
-      <c r="C28" s="24"/>
+      <c r="A28" s="152"/>
+      <c r="B28" s="31" t="s">
+        <v>268</v>
+      </c>
+      <c r="C28" s="24">
+        <v>3</v>
+      </c>
       <c r="D28" s="67"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="67"/>
-      <c r="G28" s="71"/>
+      <c r="E28" s="46" t="s">
+        <v>263</v>
+      </c>
+      <c r="F28" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="68"/>
       <c r="H28" s="23" t="s">
-        <v>261</v>
-      </c>
-      <c r="I28" s="155"/>
-    </row>
-    <row r="29" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="154"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="67"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="67"/>
-      <c r="G29" s="68"/>
-      <c r="H29" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="I29" s="155"/>
+        <v>255</v>
+      </c>
+      <c r="I28" s="153"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="155"/>
+      <c r="B29" s="156" t="s">
+        <v>260</v>
+      </c>
+      <c r="C29" s="157">
+        <v>4</v>
+      </c>
+      <c r="D29" s="158"/>
+      <c r="E29" s="159" t="s">
+        <v>263</v>
+      </c>
+      <c r="F29" s="158" t="s">
+        <v>20</v>
+      </c>
+      <c r="G29" s="160"/>
+      <c r="H29" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="I29" s="161"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="157"/>
-      <c r="B30" s="158"/>
-      <c r="C30" s="137"/>
-      <c r="D30" s="159"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="159"/>
-      <c r="G30" s="160"/>
-      <c r="H30" s="140" t="s">
-        <v>259</v>
-      </c>
-      <c r="I30" s="161"/>
+      <c r="A30" s="67"/>
+      <c r="B30" s="67"/>
+      <c r="C30" s="67"/>
+      <c r="D30" s="67"/>
+      <c r="E30" s="67"/>
+      <c r="F30" s="67"/>
+      <c r="G30" s="67"/>
+      <c r="H30" s="67"/>
+      <c r="I30" s="67"/>
     </row>
     <row r="31" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="162"/>
-      <c r="B31" s="163"/>
-      <c r="C31" s="164"/>
-      <c r="D31" s="165"/>
-      <c r="E31" s="166"/>
-      <c r="F31" s="165"/>
-      <c r="G31" s="165"/>
-      <c r="H31" s="165"/>
+      <c r="B31" s="163" t="s">
+        <v>254</v>
+      </c>
+      <c r="C31" s="30">
+        <v>4</v>
+      </c>
+      <c r="D31" s="164" t="s">
+        <v>269</v>
+      </c>
+      <c r="E31" s="165" t="s">
+        <v>270</v>
+      </c>
+      <c r="F31" s="164" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="164"/>
+      <c r="H31" s="166" t="s">
+        <v>271</v>
+      </c>
       <c r="I31" s="167"/>
     </row>
     <row r="32" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="154"/>
-      <c r="B32" s="145" t="s">
-        <v>250</v>
-      </c>
-      <c r="C32" s="24">
-        <v>2</v>
-      </c>
-      <c r="D32" s="67" t="s">
-        <v>267</v>
-      </c>
+      <c r="A32" s="152"/>
+      <c r="B32" s="23" t="s">
+        <v>272</v>
+      </c>
+      <c r="C32" s="55">
+        <v>4</v>
+      </c>
+      <c r="D32" s="67"/>
       <c r="E32" s="46" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F32" s="67" t="s">
         <v>15</v>
       </c>
       <c r="G32" s="67"/>
       <c r="H32" s="52" t="s">
-        <v>269</v>
-      </c>
-      <c r="I32" s="155"/>
+        <v>273</v>
+      </c>
+      <c r="I32" s="153"/>
     </row>
     <row r="33" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="154"/>
-      <c r="B33" s="23" t="s">
-        <v>263</v>
-      </c>
-      <c r="C33" s="55">
-        <v>3</v>
+      <c r="A33" s="152"/>
+      <c r="B33" s="143" t="s">
+        <v>274</v>
+      </c>
+      <c r="C33" s="24">
+        <v>1</v>
       </c>
       <c r="D33" s="67"/>
-      <c r="E33" s="46" t="s">
-        <v>268</v>
-      </c>
-      <c r="F33" s="67" t="s">
-        <v>15</v>
-      </c>
+      <c r="E33" s="46"/>
+      <c r="F33" s="67"/>
       <c r="G33" s="67"/>
       <c r="H33" s="52" t="s">
-        <v>270</v>
-      </c>
-      <c r="I33" s="155"/>
+        <v>273</v>
+      </c>
+      <c r="I33" s="153"/>
     </row>
     <row r="34" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="154"/>
-      <c r="B34" s="145"/>
+      <c r="A34" s="152"/>
+      <c r="B34" s="23"/>
       <c r="C34" s="24"/>
       <c r="D34" s="67"/>
-      <c r="E34" s="46"/>
+      <c r="E34" s="168"/>
       <c r="F34" s="67"/>
       <c r="G34" s="67"/>
-      <c r="H34" s="52" t="s">
+      <c r="H34" s="52"/>
+      <c r="I34" s="153"/>
+    </row>
+    <row r="35" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="152"/>
+      <c r="B35" s="52" t="s">
+        <v>275</v>
+      </c>
+      <c r="C35" s="24">
+        <v>4</v>
+      </c>
+      <c r="D35" s="67"/>
+      <c r="E35" s="46" t="s">
         <v>270</v>
       </c>
-      <c r="I34" s="155"/>
-    </row>
-    <row r="35" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="154"/>
-      <c r="B35" s="23"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="67"/>
-      <c r="E35" s="168"/>
-      <c r="F35" s="67"/>
+      <c r="F35" s="67" t="s">
+        <v>20</v>
+      </c>
       <c r="G35" s="67"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="155"/>
+      <c r="H35" s="52" t="s">
+        <v>271</v>
+      </c>
+      <c r="I35" s="153"/>
     </row>
     <row r="36" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="154"/>
-      <c r="B36" s="52" t="s">
-        <v>271</v>
+      <c r="A36" s="152"/>
+      <c r="B36" s="23" t="s">
+        <v>250</v>
       </c>
       <c r="C36" s="24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" s="67"/>
       <c r="E36" s="46" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F36" s="67" t="s">
         <v>20</v>
       </c>
       <c r="G36" s="67"/>
       <c r="H36" s="52" t="s">
-        <v>269</v>
-      </c>
-      <c r="I36" s="155"/>
-    </row>
-    <row r="37" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="154"/>
+        <v>271</v>
+      </c>
+      <c r="I36" s="153"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="170"/>
       <c r="B37" s="23" t="s">
-        <v>272</v>
-      </c>
-      <c r="C37" s="24">
-        <v>3</v>
-      </c>
-      <c r="D37" s="67"/>
+        <v>276</v>
+      </c>
+      <c r="C37" s="138">
+        <v>2</v>
+      </c>
+      <c r="D37" s="171"/>
       <c r="E37" s="46" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F37" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="G37" s="67"/>
-      <c r="H37" s="52" t="s">
-        <v>269</v>
-      </c>
-      <c r="I37" s="155"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="157"/>
-      <c r="B38" s="52" t="s">
-        <v>252</v>
-      </c>
-      <c r="C38" s="137">
-        <v>3</v>
-      </c>
-      <c r="D38" s="159"/>
-      <c r="E38" s="46" t="s">
-        <v>268</v>
-      </c>
-      <c r="F38" s="159" t="s">
-        <v>20</v>
-      </c>
-      <c r="G38" s="159"/>
-      <c r="H38" s="170" t="s">
+      <c r="G37" s="171"/>
+      <c r="H37" s="172" t="s">
         <v>32</v>
       </c>
-      <c r="I38" s="161"/>
+      <c r="I37" s="173"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="174" t="s">
+        <v>277</v>
+      </c>
+      <c r="B38" s="175"/>
+      <c r="C38" s="175"/>
+      <c r="D38" s="175"/>
+      <c r="E38" s="175"/>
+      <c r="F38" s="175"/>
+      <c r="G38" s="175"/>
+      <c r="H38" s="175"/>
+      <c r="I38" s="176"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
@@ -2965,10 +3094,11 @@
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="D8:D14"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="D16:D22"/>
-    <mergeCell ref="D23:D30"/>
-    <mergeCell ref="D32:D38"/>
+    <mergeCell ref="D15:D21"/>
+    <mergeCell ref="D22:D29"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="D31:D37"/>
+    <mergeCell ref="A38:I38"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="69" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2984,14 +3114,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K480"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.42578125"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="11.453125" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" customWidth="1"/>
-    <col min="2" max="2" width="42.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" customWidth="1"/>
+    <col min="2" max="2" width="42.7265625" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
-    <col min="6" max="6" width="24.42578125" customWidth="1"/>
-    <col min="7" max="7" width="36.5703125" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" customWidth="1"/>
+    <col min="6" max="6" width="24.453125" customWidth="1"/>
+    <col min="7" max="7" width="36.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -10673,27 +10803,27 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.42578125"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="11.453125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -10802,39 +10932,39 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.42578125"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="11.453125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" customWidth="1"/>
+    <col min="4" max="4" width="22.7265625" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="171" t="s">
-        <v>274</v>
-      </c>
-      <c r="B3" s="171" t="s">
-        <v>275</v>
-      </c>
-      <c r="C3" s="171" t="s">
-        <v>276</v>
-      </c>
-      <c r="D3" s="171" t="s">
-        <v>277</v>
-      </c>
-      <c r="E3" s="171" t="s">
-        <v>278</v>
-      </c>
-      <c r="F3" s="171" t="s">
+      <c r="A3" s="177" t="s">
         <v>279</v>
+      </c>
+      <c r="B3" s="177" t="s">
+        <v>280</v>
+      </c>
+      <c r="C3" s="177" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" s="177" t="s">
+        <v>282</v>
+      </c>
+      <c r="E3" s="177" t="s">
+        <v>283</v>
+      </c>
+      <c r="F3" s="177" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Arreglos del excel para cambios en el proyecto y permita la descarga correcta de dichos documentos
</commit_message>
<xml_diff>
--- a/facultad-derecho/tempExcels/Semana1.xlsx
+++ b/facultad-derecho/tempExcels/Semana1.xlsx
@@ -13,14 +13,14 @@
     <sheet sheetId="8" name="TURNOS ADICIONALES " state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'IMPRIMIR SEMANAL'!$A1:$I38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'IMPRIMIR SEMANAL'!$A1:$I39</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1248" uniqueCount="260">
   <si>
     <t>UNIVERSIDAD COLEGIO MAYOR DE CUNDINAMARCA</t>
   </si>
@@ -739,7 +739,7 @@
     <t>LISTADO DE ASIGNACION DE TURNOS PARA ESTUDIANTES  PERIODO  2025-II</t>
   </si>
   <si>
-    <t>SEMANA No. 17 NOVIEMBRE 19 - 21</t>
+    <t>SEMANA No. 7 SEPTIEMBRE 08-12</t>
   </si>
   <si>
     <t>APELLIDOS Y NOMBRES ESTUDIANTE</t>
@@ -766,91 +766,13 @@
     <t xml:space="preserve">LUNES </t>
   </si>
   <si>
-    <t>LINA PAOLA TRIANA MARTINEZ</t>
-  </si>
-  <si>
-    <t>ROBERTO ANGEL BADRAN BLANCO</t>
-  </si>
-  <si>
-    <t>ERICK SANTIAGO RICO LOPEZ</t>
-  </si>
-  <si>
-    <t>MIERCOLES</t>
-  </si>
-  <si>
-    <t>NOV-19,-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANDRES RICARDO MORENO SANGUINO </t>
-  </si>
-  <si>
-    <t>DAVID RICARDO JARAMILLO ZALDUA</t>
-  </si>
-  <si>
-    <t>FRANCISCO ALVARO FAJARDO PINILLA</t>
-  </si>
-  <si>
-    <t>PAULA ANDREA QUINTERO VARGAS</t>
-  </si>
-  <si>
-    <t>MORALES PERALTA VALENTINA</t>
-  </si>
-  <si>
-    <t>LEIDY NATALIA MONCADA VEGA</t>
-  </si>
-  <si>
-    <t>WILLIAM GIOVANNI MORENO AVILA</t>
-  </si>
-  <si>
-    <t>DANIEL ESTEBAN QUINTERO CARMONA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUEVES </t>
-  </si>
-  <si>
-    <t>JAIME ESTEBAN CAMARGO MENA</t>
-  </si>
-  <si>
-    <t>NOV-20,-2025</t>
-  </si>
-  <si>
-    <t>ROSEMBER SIERRA AVILA</t>
-  </si>
-  <si>
-    <t>SANTIAGO GONZALEZ VARGAS</t>
-  </si>
-  <si>
-    <t>KAROL ANDREA FLOREZ RODRIGUEZ</t>
-  </si>
-  <si>
-    <t>NICOL DAYAN JIMENEZ GUTIERREZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JONIER ALEXANDER ROJAS </t>
-  </si>
-  <si>
-    <t>VIERNES</t>
-  </si>
-  <si>
-    <t>NOV-21,-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROCIO DEL PILAR ROJAS ROCHA </t>
-  </si>
-  <si>
-    <t>TANIA SOFIA RAMIREZ MEDINA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NELSON ENRIQUE RUEDA RODRIGUEZ </t>
-  </si>
-  <si>
-    <t>KIMBERLY DANIELA GONZALES CARRERO</t>
-  </si>
-  <si>
-    <t>JIMENEZ GALVIS ISIDRO</t>
-  </si>
-  <si>
-    <t>JULIAN ESTEBAN ACERO CASTILLO</t>
+    <t>MARTES</t>
+  </si>
+  <si>
+    <t>MIÉRCOLES</t>
+  </si>
+  <si>
+    <t>JUEVES</t>
   </si>
   <si>
     <t>DÍA DE CONCILIACIONES Y/O SALIDA PEDAGOGICA</t>
@@ -1085,7 +1007,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -1419,58 +1341,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.3999755851924192"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1491,11 +1361,11 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right/>
+      <top style="medium">
         <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1503,9 +1373,37 @@
     <border>
       <left/>
       <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
-        <color theme="4" tint="0.3999755851924192"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1519,6 +1417,69 @@
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.3999755851924192"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.3999755851924192"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1548,7 +1509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1873,9 +1834,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1888,114 +1846,111 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2408,7 +2363,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="11.453125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.453125" customWidth="1"/>
@@ -2423,7 +2378,7 @@
     <col min="10" max="10" width="22.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.5" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="111" t="s">
         <v>0</v>
       </c>
@@ -2436,7 +2391,7 @@
       <c r="H1" s="112"/>
       <c r="I1" s="113"/>
     </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.5" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="114" t="s">
         <v>1</v>
       </c>
@@ -2449,7 +2404,7 @@
       <c r="H2" s="115"/>
       <c r="I2" s="116"/>
     </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.5" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="114" t="s">
         <v>2</v>
       </c>
@@ -2462,7 +2417,7 @@
       <c r="H3" s="115"/>
       <c r="I3" s="116"/>
     </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.5" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="114" t="s">
         <v>237</v>
       </c>
@@ -2475,7 +2430,7 @@
       <c r="H4" s="115"/>
       <c r="I4" s="116"/>
     </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.5" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="114" t="s">
         <v>238</v>
       </c>
@@ -2488,7 +2443,7 @@
       <c r="H5" s="115"/>
       <c r="I5" s="116"/>
     </row>
-    <row r="6" ht="16.5" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="16" customHeight="1" spans="1:9" s="110" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="117" t="s">
         <v>239</v>
       </c>
@@ -2540,553 +2495,360 @@
       <c r="E8" s="127"/>
       <c r="F8" s="126"/>
       <c r="G8" s="128"/>
-      <c r="H8" s="129" t="s">
-        <v>248</v>
-      </c>
+      <c r="H8" s="129"/>
       <c r="I8" s="130"/>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="131"/>
-      <c r="B9" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="B9" s="23"/>
       <c r="C9" s="24"/>
       <c r="D9" s="24"/>
-      <c r="E9" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="E9" s="46"/>
       <c r="F9" s="24"/>
       <c r="G9" s="25"/>
-      <c r="H9" s="23" t="s">
-        <v>248</v>
-      </c>
-      <c r="I9" s="133"/>
-    </row>
-    <row r="10" ht="15.5" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="23"/>
+      <c r="I9" s="132"/>
+    </row>
+    <row r="10" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="131"/>
-      <c r="B10" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="B10" s="23"/>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
-      <c r="E10" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="E10" s="46"/>
       <c r="F10" s="24"/>
       <c r="G10" s="25"/>
-      <c r="H10" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="I10" s="133"/>
-    </row>
-    <row r="11" ht="15.5" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H10" s="23"/>
+      <c r="I10" s="132"/>
+    </row>
+    <row r="11" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="131"/>
-      <c r="B11" s="132" t="s">
-        <v>160</v>
-      </c>
-      <c r="C11" s="134"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="133"/>
       <c r="D11" s="24"/>
-      <c r="E11" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="E11" s="46"/>
       <c r="F11" s="24"/>
       <c r="G11" s="25"/>
       <c r="H11" s="28"/>
-      <c r="I11" s="133"/>
-    </row>
-    <row r="12" ht="15.5" customHeight="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I11" s="132"/>
+    </row>
+    <row r="12" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="131"/>
-      <c r="B12" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="B12" s="23"/>
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
-      <c r="E12" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="E12" s="46"/>
       <c r="F12" s="24"/>
       <c r="G12" s="25"/>
-      <c r="H12" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="I12" s="133"/>
-      <c r="J12" s="135"/>
-    </row>
-    <row r="13" ht="15.5" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H12" s="23"/>
+      <c r="I12" s="132"/>
+      <c r="J12" s="134"/>
+    </row>
+    <row r="13" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="131"/>
-      <c r="B13" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="B13" s="23"/>
       <c r="C13" s="24"/>
       <c r="D13" s="24"/>
-      <c r="E13" s="132" t="s">
-        <v>160</v>
-      </c>
+      <c r="E13" s="46"/>
       <c r="F13" s="24"/>
       <c r="G13" s="25"/>
-      <c r="H13" s="23" t="s">
+      <c r="H13" s="23"/>
+      <c r="I13" s="132"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="135"/>
+      <c r="B14" s="136"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="137"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="138"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="139"/>
+      <c r="B15" s="140"/>
+      <c r="C15" s="140"/>
+      <c r="D15" s="140"/>
+      <c r="E15" s="140"/>
+      <c r="F15" s="140"/>
+      <c r="G15" s="140"/>
+      <c r="H15" s="140"/>
+      <c r="I15" s="141"/>
+    </row>
+    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="142"/>
+      <c r="B16" s="143"/>
+      <c r="C16" s="144"/>
+      <c r="D16" s="145" t="s">
         <v>248</v>
       </c>
-      <c r="I13" s="133"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="136"/>
-      <c r="B14" s="137"/>
-      <c r="C14" s="138"/>
-      <c r="D14" s="138"/>
-      <c r="E14" s="139"/>
-      <c r="F14" s="138"/>
-      <c r="G14" s="140"/>
-      <c r="H14" s="141" t="s">
-        <v>248</v>
-      </c>
-      <c r="I14" s="142"/>
-    </row>
-    <row r="15" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="124"/>
-      <c r="B15" s="143" t="s">
-        <v>250</v>
-      </c>
-      <c r="C15" s="144">
-        <v>1</v>
-      </c>
-      <c r="D15" s="145" t="s">
-        <v>251</v>
-      </c>
-      <c r="E15" s="127" t="s">
-        <v>252</v>
-      </c>
-      <c r="F15" s="126" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="128"/>
-      <c r="H15" s="129" t="s">
-        <v>253</v>
-      </c>
-      <c r="I15" s="130"/>
-    </row>
-    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="131"/>
-      <c r="B16" s="23" t="s">
-        <v>254</v>
-      </c>
-      <c r="C16" s="24">
-        <v>4</v>
-      </c>
-      <c r="D16" s="146"/>
-      <c r="E16" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="F16" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" s="25"/>
-      <c r="H16" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="I16" s="133"/>
+      <c r="E16" s="146"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="147"/>
+      <c r="H16" s="148"/>
+      <c r="I16" s="149"/>
     </row>
     <row r="17" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="131"/>
-      <c r="B17" s="52" t="s">
-        <v>256</v>
-      </c>
-      <c r="C17" s="24">
-        <v>3</v>
-      </c>
-      <c r="D17" s="146"/>
-      <c r="E17" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="F17" s="24" t="s">
-        <v>15</v>
-      </c>
+      <c r="B17" s="23"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="145"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="24"/>
       <c r="G17" s="25"/>
-      <c r="H17" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="I17" s="133"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="132"/>
     </row>
     <row r="18" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="131"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="134"/>
-      <c r="D18" s="146"/>
+      <c r="B18" s="52"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="145"/>
+      <c r="E18" s="46"/>
       <c r="F18" s="24"/>
       <c r="G18" s="25"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="133"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="132"/>
     </row>
     <row r="19" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="131"/>
-      <c r="B19" s="72" t="s">
-        <v>257</v>
-      </c>
-      <c r="C19" s="24">
-        <v>4</v>
-      </c>
-      <c r="D19" s="146"/>
-      <c r="E19" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="F19" s="24" t="s">
-        <v>20</v>
-      </c>
+      <c r="B19" s="23"/>
+      <c r="C19" s="133"/>
+      <c r="D19" s="145"/>
+      <c r="F19" s="24"/>
       <c r="G19" s="25"/>
-      <c r="H19" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="I19" s="133"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="132"/>
     </row>
     <row r="20" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="131"/>
-      <c r="B20" s="23" t="s">
-        <v>258</v>
-      </c>
-      <c r="C20" s="55">
-        <v>4</v>
-      </c>
-      <c r="D20" s="146"/>
-      <c r="E20" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="F20" s="24" t="s">
-        <v>20</v>
-      </c>
+      <c r="B20" s="72"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="145"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="24"/>
       <c r="G20" s="25"/>
-      <c r="H20" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="I20" s="133"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="136"/>
-      <c r="B21" s="77" t="s">
-        <v>260</v>
-      </c>
-      <c r="C21" s="147">
-        <v>4</v>
-      </c>
-      <c r="D21" s="148"/>
-      <c r="E21" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="F21" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="G21" s="140"/>
-      <c r="H21" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="I21" s="142"/>
-    </row>
-    <row r="22" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="124"/>
-      <c r="B22" s="149"/>
-      <c r="C22" s="126"/>
-      <c r="D22" s="150" t="s">
-        <v>261</v>
-      </c>
-      <c r="E22" s="151"/>
-      <c r="F22" s="126"/>
-      <c r="G22" s="126"/>
-      <c r="H22" s="129"/>
-      <c r="I22" s="130"/>
-    </row>
-    <row r="23" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H20" s="23"/>
+      <c r="I20" s="132"/>
+    </row>
+    <row r="21" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="131"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="145"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="132"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="135"/>
+      <c r="B22" s="150"/>
+      <c r="C22" s="151"/>
+      <c r="D22" s="145"/>
+      <c r="E22" s="137"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="19"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="152"/>
-      <c r="B23" s="52" t="s">
-        <v>262</v>
-      </c>
-      <c r="C23" s="24">
-        <v>1</v>
-      </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="46" t="s">
-        <v>263</v>
-      </c>
-      <c r="F23" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" s="71"/>
-      <c r="H23" s="52" t="s">
-        <v>264</v>
-      </c>
-      <c r="I23" s="153"/>
+      <c r="B23" s="153"/>
+      <c r="C23" s="153"/>
+      <c r="D23" s="153"/>
+      <c r="E23" s="153"/>
+      <c r="F23" s="153"/>
+      <c r="G23" s="153"/>
+      <c r="H23" s="153"/>
+      <c r="I23" s="154"/>
     </row>
     <row r="24" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="152"/>
-      <c r="B24" s="31" t="s">
-        <v>265</v>
-      </c>
-      <c r="C24" s="38">
-        <v>1</v>
-      </c>
-      <c r="D24" s="67"/>
-      <c r="E24" s="46" t="s">
-        <v>263</v>
-      </c>
-      <c r="F24" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="68"/>
-      <c r="H24" s="52" t="s">
-        <v>264</v>
-      </c>
-      <c r="I24" s="153"/>
+      <c r="A24" s="155"/>
+      <c r="B24" s="156"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="157" t="s">
+        <v>249</v>
+      </c>
+      <c r="E24" s="146"/>
+      <c r="F24" s="144"/>
+      <c r="G24" s="158"/>
+      <c r="H24" s="156"/>
+      <c r="I24" s="159"/>
     </row>
     <row r="25" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="152"/>
-      <c r="B25" s="125" t="s">
-        <v>266</v>
-      </c>
-      <c r="C25" s="55">
-        <v>2</v>
-      </c>
-      <c r="D25" s="67"/>
+      <c r="A25" s="160"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="157"/>
       <c r="E25" s="46"/>
       <c r="F25" s="67"/>
-      <c r="G25" s="71"/>
-      <c r="H25" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="I25" s="153"/>
+      <c r="G25" s="68"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="161"/>
     </row>
     <row r="26" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="152"/>
-      <c r="B26" s="26"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="68"/>
+      <c r="A26" s="160"/>
+      <c r="B26" s="125"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="157"/>
+      <c r="E26" s="46"/>
       <c r="F26" s="67"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="154"/>
-      <c r="I26" s="153"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="161"/>
     </row>
     <row r="27" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="152"/>
-      <c r="B27" s="77" t="s">
-        <v>267</v>
-      </c>
-      <c r="C27" s="24">
-        <v>4</v>
-      </c>
-      <c r="D27" s="67"/>
-      <c r="E27" s="46" t="s">
-        <v>263</v>
-      </c>
-      <c r="F27" s="67" t="s">
-        <v>20</v>
-      </c>
-      <c r="G27" s="71"/>
-      <c r="H27" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="I27" s="153"/>
+      <c r="A27" s="160"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="157"/>
+      <c r="E27" s="68"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="162"/>
+      <c r="I27" s="161"/>
     </row>
     <row r="28" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="152"/>
-      <c r="B28" s="31" t="s">
-        <v>268</v>
-      </c>
-      <c r="C28" s="24">
-        <v>3</v>
-      </c>
-      <c r="D28" s="67"/>
-      <c r="E28" s="46" t="s">
-        <v>263</v>
-      </c>
-      <c r="F28" s="67" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="68"/>
-      <c r="H28" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="I28" s="153"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="155"/>
-      <c r="B29" s="156" t="s">
-        <v>260</v>
-      </c>
-      <c r="C29" s="157">
-        <v>4</v>
-      </c>
-      <c r="D29" s="158"/>
-      <c r="E29" s="159" t="s">
-        <v>263</v>
-      </c>
-      <c r="F29" s="158" t="s">
-        <v>20</v>
-      </c>
-      <c r="G29" s="160"/>
-      <c r="H29" s="18" t="s">
-        <v>255</v>
-      </c>
+      <c r="A28" s="160"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="157"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="67"/>
+      <c r="G28" s="71"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="161"/>
+    </row>
+    <row r="29" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="160"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="157"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="67"/>
+      <c r="G29" s="68"/>
+      <c r="H29" s="23"/>
       <c r="I29" s="161"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="67"/>
-      <c r="B30" s="67"/>
-      <c r="C30" s="67"/>
-      <c r="D30" s="67"/>
-      <c r="E30" s="67"/>
-      <c r="F30" s="67"/>
-      <c r="G30" s="67"/>
-      <c r="H30" s="67"/>
-      <c r="I30" s="67"/>
-    </row>
-    <row r="31" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="162"/>
-      <c r="B31" s="163" t="s">
-        <v>254</v>
-      </c>
-      <c r="C31" s="30">
-        <v>4</v>
-      </c>
-      <c r="D31" s="164" t="s">
-        <v>269</v>
-      </c>
-      <c r="E31" s="165" t="s">
-        <v>270</v>
-      </c>
-      <c r="F31" s="164" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="164"/>
-      <c r="H31" s="166" t="s">
-        <v>271</v>
-      </c>
-      <c r="I31" s="167"/>
+    <row r="30" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="163"/>
+      <c r="B30" s="164"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="157"/>
+      <c r="E30" s="137"/>
+      <c r="F30" s="165"/>
+      <c r="G30" s="166"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="167"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="152"/>
+      <c r="B31" s="153"/>
+      <c r="C31" s="153"/>
+      <c r="D31" s="153"/>
+      <c r="E31" s="153"/>
+      <c r="F31" s="153"/>
+      <c r="G31" s="153"/>
+      <c r="H31" s="153"/>
+      <c r="I31" s="154"/>
     </row>
     <row r="32" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="152"/>
-      <c r="B32" s="23" t="s">
-        <v>272</v>
-      </c>
-      <c r="C32" s="55">
-        <v>4</v>
-      </c>
-      <c r="D32" s="67"/>
-      <c r="E32" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="F32" s="67" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" s="67"/>
-      <c r="H32" s="52" t="s">
-        <v>273</v>
-      </c>
-      <c r="I32" s="153"/>
+      <c r="A32" s="155"/>
+      <c r="B32" s="168"/>
+      <c r="C32" s="30"/>
+      <c r="D32" s="144" t="s">
+        <v>250</v>
+      </c>
+      <c r="E32" s="146"/>
+      <c r="F32" s="144"/>
+      <c r="G32" s="144"/>
+      <c r="H32" s="156"/>
+      <c r="I32" s="159"/>
     </row>
     <row r="33" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="152"/>
-      <c r="B33" s="143" t="s">
-        <v>274</v>
-      </c>
-      <c r="C33" s="24">
-        <v>1</v>
-      </c>
+      <c r="A33" s="160"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="55"/>
       <c r="D33" s="67"/>
       <c r="E33" s="46"/>
       <c r="F33" s="67"/>
       <c r="G33" s="67"/>
-      <c r="H33" s="52" t="s">
-        <v>273</v>
-      </c>
-      <c r="I33" s="153"/>
+      <c r="H33" s="52"/>
+      <c r="I33" s="161"/>
     </row>
     <row r="34" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="152"/>
-      <c r="B34" s="23"/>
+      <c r="A34" s="160"/>
+      <c r="B34" s="169"/>
       <c r="C34" s="24"/>
       <c r="D34" s="67"/>
-      <c r="E34" s="168"/>
+      <c r="E34" s="46"/>
       <c r="F34" s="67"/>
       <c r="G34" s="67"/>
       <c r="H34" s="52"/>
-      <c r="I34" s="153"/>
+      <c r="I34" s="161"/>
     </row>
     <row r="35" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="152"/>
-      <c r="B35" s="52" t="s">
-        <v>275</v>
-      </c>
-      <c r="C35" s="24">
-        <v>4</v>
-      </c>
+      <c r="A35" s="160"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="24"/>
       <c r="D35" s="67"/>
-      <c r="E35" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="F35" s="67" t="s">
-        <v>20</v>
-      </c>
+      <c r="E35" s="170"/>
+      <c r="F35" s="67"/>
       <c r="G35" s="67"/>
-      <c r="H35" s="52" t="s">
-        <v>271</v>
-      </c>
-      <c r="I35" s="153"/>
+      <c r="H35" s="52"/>
+      <c r="I35" s="161"/>
     </row>
     <row r="36" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="152"/>
-      <c r="B36" s="23" t="s">
-        <v>250</v>
-      </c>
-      <c r="C36" s="24">
-        <v>1</v>
-      </c>
+      <c r="A36" s="160"/>
+      <c r="B36" s="52"/>
+      <c r="C36" s="24"/>
       <c r="D36" s="67"/>
-      <c r="E36" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="F36" s="67" t="s">
-        <v>20</v>
-      </c>
+      <c r="E36" s="46"/>
+      <c r="F36" s="67"/>
       <c r="G36" s="67"/>
-      <c r="H36" s="52" t="s">
-        <v>271</v>
-      </c>
-      <c r="I36" s="153"/>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" spans="1:9" s="169" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="170"/>
-      <c r="B37" s="23" t="s">
-        <v>276</v>
-      </c>
-      <c r="C37" s="138">
-        <v>2</v>
-      </c>
-      <c r="D37" s="171"/>
-      <c r="E37" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="F37" s="67" t="s">
-        <v>20</v>
-      </c>
-      <c r="G37" s="171"/>
-      <c r="H37" s="172" t="s">
-        <v>32</v>
-      </c>
-      <c r="I37" s="173"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="174" t="s">
-        <v>277</v>
-      </c>
-      <c r="B38" s="175"/>
-      <c r="C38" s="175"/>
-      <c r="D38" s="175"/>
-      <c r="E38" s="175"/>
-      <c r="F38" s="175"/>
-      <c r="G38" s="175"/>
-      <c r="H38" s="175"/>
-      <c r="I38" s="176"/>
+      <c r="H36" s="52"/>
+      <c r="I36" s="161"/>
+    </row>
+    <row r="37" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="160"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="67"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="67"/>
+      <c r="G37" s="67"/>
+      <c r="H37" s="52"/>
+      <c r="I37" s="161"/>
+    </row>
+    <row r="38" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="67"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="67"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="67"/>
+      <c r="G38" s="67"/>
+      <c r="H38" s="52"/>
+      <c r="I38" s="67"/>
+    </row>
+    <row r="39" spans="1:9" s="171" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="172" t="s">
+        <v>251</v>
+      </c>
+      <c r="B39" s="173"/>
+      <c r="C39" s="173"/>
+      <c r="D39" s="173"/>
+      <c r="E39" s="173"/>
+      <c r="F39" s="173"/>
+      <c r="G39" s="173"/>
+      <c r="H39" s="173"/>
+      <c r="I39" s="174"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
@@ -3094,11 +2856,13 @@
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="D8:D14"/>
-    <mergeCell ref="D15:D21"/>
-    <mergeCell ref="D22:D29"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="D31:D37"/>
-    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="D16:D22"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="D24:D30"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="D32:D38"/>
+    <mergeCell ref="A39:I39"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="69" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -3124,7 +2888,7 @@
     <col min="7" max="7" width="36.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="18.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3135,7 +2899,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" ht="18.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -3146,7 +2910,7 @@
       <c r="F2" s="6"/>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" ht="18.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -3157,7 +2921,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="7"/>
     </row>
-    <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" ht="18.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
@@ -3168,7 +2932,7 @@
       <c r="F4" s="6"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" ht="18.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -6402,7 +6166,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="168" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="45">
         <v>162</v>
       </c>
@@ -10812,18 +10576,18 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>285</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>279</v>
+        <v>253</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>280</v>
+        <v>254</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>281</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -10944,27 +10708,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>278</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="177" t="s">
-        <v>279</v>
-      </c>
-      <c r="B3" s="177" t="s">
-        <v>280</v>
-      </c>
-      <c r="C3" s="177" t="s">
-        <v>281</v>
-      </c>
-      <c r="D3" s="177" t="s">
-        <v>282</v>
-      </c>
-      <c r="E3" s="177" t="s">
-        <v>283</v>
-      </c>
-      <c r="F3" s="177" t="s">
-        <v>284</v>
+      <c r="A3" s="175" t="s">
+        <v>253</v>
+      </c>
+      <c r="B3" s="175" t="s">
+        <v>254</v>
+      </c>
+      <c r="C3" s="175" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" s="175" t="s">
+        <v>256</v>
+      </c>
+      <c r="E3" s="175" t="s">
+        <v>257</v>
+      </c>
+      <c r="F3" s="175" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Implementaciones de seguridad para la mejora de horario
</commit_message>
<xml_diff>
--- a/facultad-derecho/tempExcels/Semana1.xlsx
+++ b/facultad-derecho/tempExcels/Semana1.xlsx
@@ -13,7 +13,7 @@
     <sheet sheetId="8" name="TURNOS ADICIONALES " state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'IMPRIMIR SEMANAL'!$A1:$I39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'IMPRIMIR SEMANAL'!$A1:$I38</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
@@ -736,10 +736,10 @@
     <t>SEDE. CONVENIO UPK -TINTAL "UNIVERSIDAD PÚBLICA EN KENNEDY"</t>
   </si>
   <si>
-    <t>LISTADO DE ASIGNACION DE TURNOS PARA ESTUDIANTES  PERIODO  2025-II</t>
-  </si>
-  <si>
-    <t>SEMANA No. 7 SEPTIEMBRE 08-12</t>
+    <t>LISTADO DE ASIGNACION DE TURNOS PARA ESTUDIANTES  PERIODO  2026 - S1</t>
+  </si>
+  <si>
+    <t>SEMANA No. 1</t>
   </si>
   <si>
     <t>APELLIDOS Y NOMBRES ESTUDIANTE</t>
@@ -769,13 +769,13 @@
     <t>MARTES</t>
   </si>
   <si>
-    <t>MIÉRCOLES</t>
-  </si>
-  <si>
-    <t>JUEVES</t>
-  </si>
-  <si>
     <t>DÍA DE CONCILIACIONES Y/O SALIDA PEDAGOGICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JUEVES </t>
+  </si>
+  <si>
+    <t>VIERNES</t>
   </si>
   <si>
     <t xml:space="preserve">MODIFICACION  DE TURNOS </t>
@@ -1436,27 +1436,8 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1466,12 +1447,8 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1490,8 +1467,25 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1501,15 +1495,19 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1888,13 +1886,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1932,7 +1930,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1944,13 +1942,20 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2363,7 +2368,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="11.453125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.453125" customWidth="1"/>
@@ -2643,19 +2648,21 @@
       <c r="H21" s="23"/>
       <c r="I21" s="132"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="135"/>
       <c r="B22" s="150"/>
       <c r="C22" s="151"/>
       <c r="D22" s="145"/>
-      <c r="E22" s="137"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="19"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="152"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="24"/>
+    </row>
+    <row r="23" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="152" t="s">
+        <v>249</v>
+      </c>
       <c r="B23" s="153"/>
       <c r="C23" s="153"/>
       <c r="D23" s="153"/>
@@ -2670,7 +2677,7 @@
       <c r="B24" s="156"/>
       <c r="C24" s="30"/>
       <c r="D24" s="157" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E24" s="146"/>
       <c r="F24" s="144"/>
@@ -2745,22 +2752,22 @@
       <c r="I30" s="167"/>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="152"/>
-      <c r="B31" s="153"/>
-      <c r="C31" s="153"/>
-      <c r="D31" s="153"/>
-      <c r="E31" s="153"/>
-      <c r="F31" s="153"/>
-      <c r="G31" s="153"/>
-      <c r="H31" s="153"/>
-      <c r="I31" s="154"/>
+      <c r="A31" s="139"/>
+      <c r="B31" s="140"/>
+      <c r="C31" s="140"/>
+      <c r="D31" s="140"/>
+      <c r="E31" s="140"/>
+      <c r="F31" s="140"/>
+      <c r="G31" s="140"/>
+      <c r="H31" s="140"/>
+      <c r="I31" s="141"/>
     </row>
     <row r="32" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="155"/>
       <c r="B32" s="168"/>
       <c r="C32" s="30"/>
-      <c r="D32" s="144" t="s">
-        <v>250</v>
+      <c r="D32" s="157" t="s">
+        <v>251</v>
       </c>
       <c r="E32" s="146"/>
       <c r="F32" s="144"/>
@@ -2772,7 +2779,7 @@
       <c r="A33" s="160"/>
       <c r="B33" s="23"/>
       <c r="C33" s="55"/>
-      <c r="D33" s="67"/>
+      <c r="D33" s="157"/>
       <c r="E33" s="46"/>
       <c r="F33" s="67"/>
       <c r="G33" s="67"/>
@@ -2783,7 +2790,7 @@
       <c r="A34" s="160"/>
       <c r="B34" s="169"/>
       <c r="C34" s="24"/>
-      <c r="D34" s="67"/>
+      <c r="D34" s="157"/>
       <c r="E34" s="46"/>
       <c r="F34" s="67"/>
       <c r="G34" s="67"/>
@@ -2794,7 +2801,7 @@
       <c r="A35" s="160"/>
       <c r="B35" s="23"/>
       <c r="C35" s="24"/>
-      <c r="D35" s="67"/>
+      <c r="D35" s="157"/>
       <c r="E35" s="170"/>
       <c r="F35" s="67"/>
       <c r="G35" s="67"/>
@@ -2805,7 +2812,7 @@
       <c r="A36" s="160"/>
       <c r="B36" s="52"/>
       <c r="C36" s="24"/>
-      <c r="D36" s="67"/>
+      <c r="D36" s="157"/>
       <c r="E36" s="46"/>
       <c r="F36" s="67"/>
       <c r="G36" s="67"/>
@@ -2816,39 +2823,26 @@
       <c r="A37" s="160"/>
       <c r="B37" s="23"/>
       <c r="C37" s="24"/>
-      <c r="D37" s="67"/>
+      <c r="D37" s="157"/>
       <c r="E37" s="46"/>
       <c r="F37" s="67"/>
       <c r="G37" s="67"/>
       <c r="H37" s="52"/>
       <c r="I37" s="161"/>
     </row>
-    <row r="38" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="67"/>
-      <c r="B38" s="23"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="67"/>
+    <row r="38" ht="15" customHeight="1" spans="1:9" s="171" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="172"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="173"/>
+      <c r="D38" s="174"/>
       <c r="E38" s="46"/>
-      <c r="F38" s="67"/>
-      <c r="G38" s="67"/>
-      <c r="H38" s="52"/>
-      <c r="I38" s="67"/>
-    </row>
-    <row r="39" spans="1:9" s="171" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="172" t="s">
-        <v>251</v>
-      </c>
-      <c r="B39" s="173"/>
-      <c r="C39" s="173"/>
-      <c r="D39" s="173"/>
-      <c r="E39" s="173"/>
-      <c r="F39" s="173"/>
-      <c r="G39" s="173"/>
-      <c r="H39" s="173"/>
-      <c r="I39" s="174"/>
+      <c r="F38" s="175"/>
+      <c r="G38" s="175"/>
+      <c r="H38" s="176"/>
+      <c r="I38" s="177"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
@@ -2862,7 +2856,6 @@
     <mergeCell ref="D24:D30"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="D32:D38"/>
-    <mergeCell ref="A39:I39"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="69" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -10712,22 +10705,22 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="175" t="s">
+      <c r="A3" s="178" t="s">
         <v>253</v>
       </c>
-      <c r="B3" s="175" t="s">
+      <c r="B3" s="178" t="s">
         <v>254</v>
       </c>
-      <c r="C3" s="175" t="s">
+      <c r="C3" s="178" t="s">
         <v>255</v>
       </c>
-      <c r="D3" s="175" t="s">
+      <c r="D3" s="178" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="175" t="s">
+      <c r="E3" s="178" t="s">
         <v>257</v>
       </c>
-      <c r="F3" s="175" t="s">
+      <c r="F3" s="178" t="s">
         <v>258</v>
       </c>
     </row>

</xml_diff>